<commit_message>
Refactor dashboard layout and simplify application workflows
</commit_message>
<xml_diff>
--- a/dados/enviadas/Air Liquide.xlsx
+++ b/dados/enviadas/Air Liquide.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$J$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -451,18 +451,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="59" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,35 +479,40 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>MODALIDADE</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>VALOR_ESTIMADO</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>ORGAO</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>DATA_DISPUTA</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>PORTAL</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>LINK_PORTAL</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>LINK_PNCP</t>
         </is>
@@ -520,40 +526,45 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>43/2026</t>
+          <t>18/2026</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>Gases medicinais</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>1592091.84</v>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DA LAPA</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>31/08/2026</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>ComprasGov</t>
+      <c r="E2" s="4" t="n">
+        <v>1318511</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE PALMEIRA DOS INDIOS</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98765705000432026</t>
+          <t>BNC Compras</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/76020452000105/2026/210</t>
+          <t>https://bnccompras.com/Process/ProcessView?param1=[gkz]NFPHH/QXuB7hsDwpeL_0vVEtRbHJctaLMmIxe_r6hhdfANlQaYCPMAHwTBDPVx9HZ5LgVmxDUCovg4WE7N2emF3Bw4VcR_3I37uT9qO7Qdo=</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/12356879000198/2026/92</t>
         </is>
       </c>
     </row>
@@ -565,40 +576,45 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>00018/2026</t>
+          <t>0000054/2026</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t>Oxigênio medicinal</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>384942.4</v>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE ALMENARA</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>26/08/2026</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>BNC Compras</t>
+      <c r="E3" s="4" t="n">
+        <v>91512</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE SERTAOZINHO</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>https://bnccompras.com/Process/ProcessView?param1=[gkz]AznpS838rYmU0b_1fYnILyxief5mQL/ygJz7KgzQOIYx3p0StAQCKm_doZhpiXWuj5yLMrItJRjLq7uXmLWJxrr_FJG3e5yD/6i_2Fo4WJU=</t>
+          <t>BLL Compras</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/app/editais/18349894000195/2026/52</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]Bk3O9RTdv5K7mF4j3usj4mqG1ehmfbRHuq0o5dnwoRz93re4VBppywCybWT5tYcJvaw3oUD/nzc8BgW1suKPeoBNngFxDwD4vtVMvH1DXN0=</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/45371820000128/2026/270</t>
         </is>
       </c>
     </row>
@@ -610,42 +626,41 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>P.E 021/2026</t>
+          <t>DL017/2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Oxigênio medicinal</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Sigiloso</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE IBIRAPITANGA</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>25/08/2026</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>BNC Compras</t>
+          <t>Dispensa</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>13050</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>FUNDO MUNICIPAL DE SAUDE DE CERRO NEGRO</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>https://bnccompras.com/Process/ProcessView?param1=[gkz]_Y/QoE19bqFD3Cgse4MCf9TxLzVA77_EwEWrqEmzjYDK3fnUmXpMnmSd03OGC7ekHPwsWbfe4amK4jl3pVIwnq5JYvYT9gqCduSggL4F9x0=</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/13846753000164/2026/77</t>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/11430842000108/2026/24</t>
         </is>
       </c>
     </row>
@@ -657,45 +672,530 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>041/2026</t>
+          <t>102/2026</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>Oxigênio medicinal</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t>Pregão - Eletrônico</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
-        <v>166409.5</v>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE PADRE PARAISO</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>26/08/2026</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Licitar Digital</t>
+      <c r="E5" s="4" t="n">
+        <v>113812.35</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE MARILIA</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://app2.licitardigital.com.br/pesquisa/107077</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>https://pncp.gov.br/app/editais/18404764000108/2026/51</t>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/44477909000100/2026/874</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>29/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Oxigênio medicinal</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>113812.35</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE MARILIA</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>ComprasGov</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98668105000292026</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/44477909000100/2026/875</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>00030/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Oxigênio medicinal</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Sigiloso</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE ANTONIO MARTINS</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>09/10/2026</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/08348989000130/2026/35</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SMS-033/2026/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Gases medicinais</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>275450</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE PIRAI</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/29141322000132/2026/243</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>PCE 52/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Oxigênio</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>33982.55</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE MARIPA</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/95583571000102/2026/140</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>32/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Nitrogênio liquido</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>37800</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>UNIVERSIDADE ESTADUAL PAULISTA JULIO DE MESQUITA FILHO</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>ComprasGov</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=10230705000322026</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/48031918000124/2026/2610</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>17/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Oxigênio</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Sigiloso</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE AROEIRAS</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Portal de Compras Públicas</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.portaldecompraspublicas.com.br/processos/PB/Prefeitura-Municipal-de-Aroeiras-2115/PE-17-2026-2026-514471</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/08865636000108/2026/35</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>36/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Ar comprimido</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>20408</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE TERRA ROXA</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>ComprasGov</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98792105000362026</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/75587204000170/2026/249</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>PCE1908120260084/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Gases industriais</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Dispensa</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>8994</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>FUNDO ESTADUAL DE SAUDE DO ESTADO DA BAHIA</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/05816630000152/2026/7220</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>PDE 20/2026</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Oxigênio gasoso</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Dispensa</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>37970.7</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE GRAVATAL</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/82926569000147/2026/177</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>070/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Gases medicinais</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Pregão - Eletrônico</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>5552896.32</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE CAXIAS</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Portal de Compras Públicas</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.portaldecompraspublicas.com.br/processos/MA/Prefeitura-Municipal-de-Caxias-1212/PE-070-2026-2026-514499</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/app/editais/06082820000156/2026/105</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
+  <autoFilter ref="A1:J15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>